<commit_message>
+ Fix bug skill of LittleWhiteDragon
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="9" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" state="visible" r:id="rId1"/>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="E20" s="39" t="inlineStr">
         <is>
-          <t>0.8, 1, 1.2</t>
+          <t>0.7, 0.8, 0.9</t>
         </is>
       </c>
       <c r="F20" s="39" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="E21" s="39" t="inlineStr">
         <is>
-          <t>1, 1.5, 1.5</t>
+          <t>0.8, 1.0, 1.1</t>
         </is>
       </c>
       <c r="F21" s="39" t="inlineStr">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="E22" s="39" t="inlineStr">
         <is>
-          <t>1.5, 1.8, 1.8</t>
+          <t>1.2, 1.4, 1.5</t>
         </is>
       </c>
       <c r="F22" s="39" t="inlineStr">
@@ -24978,7 +24978,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="34" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="I14" s="34" t="n">
         <v>1</v>

</xml_diff>